<commit_message>
Fixed the context hand-off
</commit_message>
<xml_diff>
--- a/WorkBot/refactor/data/orders/Coffee Depot LLC/Coffee Depot LLC_Bakery_2025-10-25.xlsx
+++ b/WorkBot/refactor/data/orders/Coffee Depot LLC/Coffee Depot LLC_Bakery_2025-10-25.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +466,121 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Monin - Turmeric</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monin - Toffee Nut</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Monin - Peppermint</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Monin - Lavender</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Monin - Caramel Apple Butter</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>9.00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>90.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>